<commit_message>
research: review 34 candidate support relations and classify 69 review issues
</commit_message>
<xml_diff>
--- a/stage4_competency_graph/output/02_能力图谱关系总表.xlsx
+++ b/stage4_competency_graph/output/02_能力图谱关系总表.xlsx
@@ -21354,7 +21354,7 @@
       </c>
       <c r="P238" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只在问题记录和修正规则已给定时支持UPDATE实施；不涵盖问题识别、清洗规则设计及清洗结果验证。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q238" t="b">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="P239" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只支持给定清洗条件的记录定位；不证明完整清洗流程、异常判断及前后质量验证已安排。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q239" t="b">
@@ -22470,7 +22470,7 @@
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>第5页明确主键作用及语法；仅在关系表标识方案已确定时支持实现表达，不能把约束SQL实现等同完整模式设计。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q250" t="b">
@@ -22563,7 +22563,7 @@
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>第5页明确外键作用及语法；仅在参照关系方案已确定时支持实现，不替代实体关系识别与完整结构设计。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q251" t="b">
@@ -22842,7 +22842,7 @@
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只支持选定索引方案的创建实施，不证明能根据查询需求选择索引或验证调整收益。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q254" t="b">
@@ -22935,7 +22935,7 @@
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只支持既定方案的索引添加实施；索引选择、负面影响分析及迭代调整仍需其他依据。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q255" t="b">
@@ -23028,7 +23028,7 @@
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只在建表时定义索引的方案下成立，不代表能调整已有库索引，也不证明完整选择与调整能力。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q256" t="b">
@@ -23121,7 +23121,7 @@
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>删除/维护索引操作不等于诊断索引问题；具体变更理由与效果核查仍未由本知识单独覆盖。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q257" t="b">
@@ -23214,7 +23214,7 @@
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>第11页仅明示有无索引查询效果对比；K3指与其他索引知识组合的观察线索，不证明完整方案选择及迭代调整闭环。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q258" t="b">
@@ -23586,7 +23586,7 @@
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>在已有质量检查条件的前提下，支持筛选待核查记录；不涵盖质量维度定义、规则制定、异常原因判断和完整核查结果验证。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q262" t="b">
@@ -23772,7 +23772,7 @@
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>仅对应内外连接语法及关联条件；完整业务语义、重复行及结果正确性仍需任务情境核查。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q264" t="b">
@@ -23865,7 +23865,7 @@
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>一般SELECT只提供表达框架，不自动支持连接条件设计或多表结果核验。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q265" t="b">
@@ -23910,7 +23910,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -23940,7 +23940,7 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>外键知识帮助理解关联字段；连接并不要求存在外键约束</t>
+          <t>第5页外键约束知识仅在参照关系解释场景中帮助理解关联字段；JOIN本身不依赖外键定义，因此采用条件性K4而非一般基础前提。</t>
         </is>
       </c>
       <c r="M266" t="inlineStr">
@@ -23958,7 +23958,7 @@
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>外键知识仅在解释既有参照关系时提供条件性理解线索；SQL JOIN不要求已定义外键约束，不是必要前提。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q266" t="b">
@@ -39356,7 +39356,7 @@
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只在问题记录和修正规则已给定时支持UPDATE实施；不涵盖问题识别、清洗规则设计及清洗结果验证。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q178" t="b">
@@ -39449,7 +39449,7 @@
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只支持给定清洗条件的记录定位；不证明完整清洗流程、异常判断及前后质量验证已安排。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q179" t="b">
@@ -40472,7 +40472,7 @@
       </c>
       <c r="P190" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>第5页明确主键作用及语法；仅在关系表标识方案已确定时支持实现表达，不能把约束SQL实现等同完整模式设计。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q190" t="b">
@@ -40565,7 +40565,7 @@
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>第5页明确外键作用及语法；仅在参照关系方案已确定时支持实现，不替代实体关系识别与完整结构设计。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q191" t="b">
@@ -40844,7 +40844,7 @@
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只支持选定索引方案的创建实施，不证明能根据查询需求选择索引或验证调整收益。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q194" t="b">
@@ -40937,7 +40937,7 @@
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只支持既定方案的索引添加实施；索引选择、负面影响分析及迭代调整仍需其他依据。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q195" t="b">
@@ -41030,7 +41030,7 @@
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>只在建表时定义索引的方案下成立，不代表能调整已有库索引，也不证明完整选择与调整能力。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q196" t="b">
@@ -41123,7 +41123,7 @@
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>删除/维护索引操作不等于诊断索引问题；具体变更理由与效果核查仍未由本知识单独覆盖。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q197" t="b">
@@ -41216,7 +41216,7 @@
       </c>
       <c r="P198" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>第11页仅明示有无索引查询效果对比；K3指与其他索引知识组合的观察线索，不证明完整方案选择及迭代调整闭环。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q198" t="b">
@@ -41588,7 +41588,7 @@
       </c>
       <c r="P202" t="inlineStr">
         <is>
-          <t>只在所述技术方案或规则已确定时适用；仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>在已有质量检查条件的前提下，支持筛选待核查记录；不涵盖质量维度定义、规则制定、异常原因判断和完整核查结果验证。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q202" t="b">
@@ -41774,7 +41774,7 @@
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>仅对应内外连接语法及关联条件；完整业务语义、重复行及结果正确性仍需任务情境核查。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q204" t="b">
@@ -41867,7 +41867,7 @@
       </c>
       <c r="P205" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>一般SELECT只提供表达框架，不自动支持连接条件设计或多表结果核验。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q205" t="b">
@@ -41912,7 +41912,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -41942,7 +41942,7 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>外键知识帮助理解关联字段；连接并不要求存在外键约束</t>
+          <t>第5页外键约束知识仅在参照关系解释场景中帮助理解关联字段；JOIN本身不依赖外键定义，因此采用条件性K4而非一般基础前提。</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
@@ -41960,7 +41960,7 @@
       </c>
       <c r="P206" t="inlineStr">
         <is>
-          <t>仅为具体技术行为支撑候选；未证明完整岗位能力已培养、学生达标或已有正式考核。</t>
+          <t>外键知识仅在解释既有参照关系时提供条件性理解线索；SQL JOIN不要求已定义外键约束，不是必要前提。 本条仍为跨体系研究推断，待人工确认。</t>
         </is>
       </c>
       <c r="Q206" t="b">

</xml_diff>